<commit_message>
Corrigindo nome da coluna no Excel base
</commit_message>
<xml_diff>
--- a/historico_beneficiarios_base.xlsx
+++ b/historico_beneficiarios_base.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://abramge-my.sharepoint.com/personal/bruno_santos_abramge_com_br/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\abramgesinogdiretoria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{C447A6D9-9569-4BE2-9231-BEEE8542EAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47F4CDAC-8B8F-4A23-AD05-0491E91CC01A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1073E1-216A-49F3-8DED-6EBD17349D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{0470967A-67BA-46B0-8E62-1A22D2427886}"/>
   </bookViews>
@@ -53,9 +53,6 @@
     <t>Porte</t>
   </si>
   <si>
-    <t>Beneficiarios ativos</t>
-  </si>
-  <si>
     <t>ASSISTÊNCIA MÉDICA</t>
   </si>
   <si>
@@ -90,6 +87,9 @@
   </si>
   <si>
     <t>ODONTOLOGIA DE GRUPO</t>
+  </si>
+  <si>
+    <t>Beneficiarios_ativos</t>
   </si>
 </sst>
 </file>
@@ -486,7 +486,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
@@ -494,13 +494,13 @@
         <v>45717</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2">
         <v>583256</v>
@@ -511,13 +511,13 @@
         <v>45717</v>
       </c>
       <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3">
         <v>978535</v>
@@ -528,13 +528,13 @@
         <v>45717</v>
       </c>
       <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4">
         <v>3009366</v>
@@ -545,13 +545,13 @@
         <v>45717</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5">
         <v>1027683</v>
@@ -562,13 +562,13 @@
         <v>45717</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6">
         <v>5104157</v>
@@ -579,13 +579,13 @@
         <v>45717</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7">
         <v>12733084</v>
@@ -596,13 +596,13 @@
         <v>45717</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8">
         <v>928144</v>
@@ -613,13 +613,13 @@
         <v>45717</v>
       </c>
       <c r="B9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9">
         <v>3071240</v>
@@ -630,13 +630,13 @@
         <v>45717</v>
       </c>
       <c r="B10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10">
         <v>16704551</v>
@@ -647,13 +647,13 @@
         <v>45717</v>
       </c>
       <c r="B11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E11">
         <v>7534</v>
@@ -664,13 +664,13 @@
         <v>45717</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12">
         <v>33640</v>
@@ -681,13 +681,13 @@
         <v>45717</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13">
         <v>6801221</v>
@@ -698,13 +698,13 @@
         <v>45717</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E14">
         <v>174980</v>
@@ -715,13 +715,13 @@
         <v>45717</v>
       </c>
       <c r="B15" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15">
         <v>529902</v>
@@ -732,13 +732,13 @@
         <v>45717</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E16">
         <v>376015</v>
@@ -749,13 +749,13 @@
         <v>45717</v>
       </c>
       <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" t="s">
         <v>14</v>
       </c>
-      <c r="C17" t="s">
-        <v>15</v>
-      </c>
       <c r="D17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17">
         <v>424033</v>
@@ -766,13 +766,13 @@
         <v>45717</v>
       </c>
       <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
         <v>14</v>
       </c>
-      <c r="C18" t="s">
-        <v>15</v>
-      </c>
       <c r="D18" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18">
         <v>1271953</v>
@@ -783,13 +783,13 @@
         <v>45717</v>
       </c>
       <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
         <v>14</v>
       </c>
-      <c r="C19" t="s">
-        <v>15</v>
-      </c>
       <c r="D19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19">
         <v>2767046</v>
@@ -800,13 +800,13 @@
         <v>45717</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D20" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E20">
         <v>494871</v>
@@ -817,13 +817,13 @@
         <v>45717</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E21">
         <v>848378</v>
@@ -834,13 +834,13 @@
         <v>45717</v>
       </c>
       <c r="B22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E22">
         <v>13905102</v>
@@ -851,13 +851,13 @@
         <v>45748</v>
       </c>
       <c r="B23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
         <v>5</v>
       </c>
-      <c r="C23" t="s">
-        <v>6</v>
-      </c>
       <c r="D23" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E23">
         <v>582071</v>
@@ -868,13 +868,13 @@
         <v>45748</v>
       </c>
       <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
         <v>5</v>
       </c>
-      <c r="C24" t="s">
-        <v>6</v>
-      </c>
       <c r="D24" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E24">
         <v>979021</v>
@@ -885,13 +885,13 @@
         <v>45748</v>
       </c>
       <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
         <v>5</v>
       </c>
-      <c r="C25" t="s">
-        <v>6</v>
-      </c>
       <c r="D25" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25">
         <v>3004900</v>
@@ -902,13 +902,13 @@
         <v>45748</v>
       </c>
       <c r="B26" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D26" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E26">
         <v>1030654</v>
@@ -919,13 +919,13 @@
         <v>45748</v>
       </c>
       <c r="B27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E27">
         <v>4904716</v>
@@ -936,13 +936,13 @@
         <v>45748</v>
       </c>
       <c r="B28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D28" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28">
         <v>12920539</v>
@@ -953,13 +953,13 @@
         <v>45748</v>
       </c>
       <c r="B29" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E29">
         <v>945390</v>
@@ -970,13 +970,13 @@
         <v>45748</v>
       </c>
       <c r="B30" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E30">
         <v>3068030</v>
@@ -987,13 +987,13 @@
         <v>45748</v>
       </c>
       <c r="B31" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C31" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E31">
         <v>16739827</v>
@@ -1004,13 +1004,13 @@
         <v>45748</v>
       </c>
       <c r="B32" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D32" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E32">
         <v>7493</v>
@@ -1021,13 +1021,13 @@
         <v>45748</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D33" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E33">
         <v>31438</v>
@@ -1038,13 +1038,13 @@
         <v>45748</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34">
         <v>6833593</v>
@@ -1055,13 +1055,13 @@
         <v>45748</v>
       </c>
       <c r="B35" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E35">
         <v>176161</v>
@@ -1072,13 +1072,13 @@
         <v>45748</v>
       </c>
       <c r="B36" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E36">
         <v>529472</v>
@@ -1089,13 +1089,13 @@
         <v>45748</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E37">
         <v>372957</v>
@@ -1106,13 +1106,13 @@
         <v>45748</v>
       </c>
       <c r="B38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" t="s">
         <v>14</v>
       </c>
-      <c r="C38" t="s">
-        <v>15</v>
-      </c>
       <c r="D38" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E38">
         <v>424140</v>
@@ -1123,13 +1123,13 @@
         <v>45748</v>
       </c>
       <c r="B39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" t="s">
         <v>14</v>
       </c>
-      <c r="C39" t="s">
-        <v>15</v>
-      </c>
       <c r="D39" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E39">
         <v>1278161</v>
@@ -1140,13 +1140,13 @@
         <v>45748</v>
       </c>
       <c r="B40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" t="s">
         <v>14</v>
       </c>
-      <c r="C40" t="s">
-        <v>15</v>
-      </c>
       <c r="D40" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E40">
         <v>2772007</v>
@@ -1157,13 +1157,13 @@
         <v>45748</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C41" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D41" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E41">
         <v>497566</v>
@@ -1174,13 +1174,13 @@
         <v>45748</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C42" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D42" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E42">
         <v>846091</v>
@@ -1191,13 +1191,13 @@
         <v>45748</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D43" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E43">
         <v>13887774</v>
@@ -1208,13 +1208,13 @@
         <v>45778</v>
       </c>
       <c r="B44" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" t="s">
         <v>5</v>
       </c>
-      <c r="C44" t="s">
-        <v>6</v>
-      </c>
       <c r="D44" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E44">
         <v>580653</v>
@@ -1225,13 +1225,13 @@
         <v>45778</v>
       </c>
       <c r="B45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
         <v>5</v>
       </c>
-      <c r="C45" t="s">
-        <v>6</v>
-      </c>
       <c r="D45" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E45">
         <v>977929</v>
@@ -1242,13 +1242,13 @@
         <v>45778</v>
       </c>
       <c r="B46" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" t="s">
         <v>5</v>
       </c>
-      <c r="C46" t="s">
-        <v>6</v>
-      </c>
       <c r="D46" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E46">
         <v>3006236</v>
@@ -1259,13 +1259,13 @@
         <v>45778</v>
       </c>
       <c r="B47" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E47">
         <v>1011813</v>
@@ -1276,13 +1276,13 @@
         <v>45778</v>
       </c>
       <c r="B48" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D48" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E48">
         <v>4928904</v>
@@ -1293,13 +1293,13 @@
         <v>45778</v>
       </c>
       <c r="B49" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C49" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D49" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E49">
         <v>12916844</v>
@@ -1310,13 +1310,13 @@
         <v>45778</v>
       </c>
       <c r="B50" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E50">
         <v>951393</v>
@@ -1327,13 +1327,13 @@
         <v>45778</v>
       </c>
       <c r="B51" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D51" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E51">
         <v>3089355</v>
@@ -1344,13 +1344,13 @@
         <v>45778</v>
       </c>
       <c r="B52" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D52" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E52">
         <v>16838527</v>
@@ -1361,13 +1361,13 @@
         <v>45778</v>
       </c>
       <c r="B53" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D53" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E53">
         <v>7460</v>
@@ -1378,13 +1378,13 @@
         <v>45778</v>
       </c>
       <c r="B54" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C54" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D54" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E54">
         <v>30939</v>
@@ -1395,13 +1395,13 @@
         <v>45778</v>
       </c>
       <c r="B55" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D55" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E55">
         <v>6892701</v>
@@ -1412,13 +1412,13 @@
         <v>45778</v>
       </c>
       <c r="B56" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D56" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E56">
         <v>177042</v>
@@ -1429,13 +1429,13 @@
         <v>45778</v>
       </c>
       <c r="B57" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D57" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E57">
         <v>532410</v>
@@ -1446,13 +1446,13 @@
         <v>45778</v>
       </c>
       <c r="B58" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D58" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E58">
         <v>371522</v>
@@ -1463,13 +1463,13 @@
         <v>45778</v>
       </c>
       <c r="B59" t="s">
+        <v>13</v>
+      </c>
+      <c r="C59" t="s">
         <v>14</v>
       </c>
-      <c r="C59" t="s">
-        <v>15</v>
-      </c>
       <c r="D59" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E59">
         <v>425200</v>
@@ -1480,13 +1480,13 @@
         <v>45778</v>
       </c>
       <c r="B60" t="s">
+        <v>13</v>
+      </c>
+      <c r="C60" t="s">
         <v>14</v>
       </c>
-      <c r="C60" t="s">
-        <v>15</v>
-      </c>
       <c r="D60" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E60">
         <v>1283470</v>
@@ -1497,13 +1497,13 @@
         <v>45778</v>
       </c>
       <c r="B61" t="s">
+        <v>13</v>
+      </c>
+      <c r="C61" t="s">
         <v>14</v>
       </c>
-      <c r="C61" t="s">
-        <v>15</v>
-      </c>
       <c r="D61" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E61">
         <v>2793013</v>
@@ -1514,13 +1514,13 @@
         <v>45778</v>
       </c>
       <c r="B62" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C62" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D62" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E62">
         <v>492129</v>
@@ -1531,13 +1531,13 @@
         <v>45778</v>
       </c>
       <c r="B63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C63" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D63" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E63">
         <v>844566</v>
@@ -1548,13 +1548,13 @@
         <v>45778</v>
       </c>
       <c r="B64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C64" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D64" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E64">
         <v>13615794</v>
@@ -1565,13 +1565,13 @@
         <v>45809</v>
       </c>
       <c r="B65" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" t="s">
         <v>5</v>
       </c>
-      <c r="C65" t="s">
-        <v>6</v>
-      </c>
       <c r="D65" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E65">
         <v>577619</v>
@@ -1582,13 +1582,13 @@
         <v>45809</v>
       </c>
       <c r="B66" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" t="s">
         <v>5</v>
       </c>
-      <c r="C66" t="s">
-        <v>6</v>
-      </c>
       <c r="D66" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E66">
         <v>975592</v>
@@ -1599,13 +1599,13 @@
         <v>45809</v>
       </c>
       <c r="B67" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" t="s">
         <v>5</v>
       </c>
-      <c r="C67" t="s">
-        <v>6</v>
-      </c>
       <c r="D67" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E67">
         <v>3006896</v>
@@ -1616,13 +1616,13 @@
         <v>45809</v>
       </c>
       <c r="B68" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D68" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E68">
         <v>1013512</v>
@@ -1633,13 +1633,13 @@
         <v>45809</v>
       </c>
       <c r="B69" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D69" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E69">
         <v>4942370</v>
@@ -1650,13 +1650,13 @@
         <v>45809</v>
       </c>
       <c r="B70" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D70" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E70">
         <v>12899773</v>
@@ -1667,13 +1667,13 @@
         <v>45809</v>
       </c>
       <c r="B71" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C71" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D71" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E71">
         <v>911543</v>
@@ -1684,13 +1684,13 @@
         <v>45809</v>
       </c>
       <c r="B72" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C72" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D72" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E72">
         <v>3203316</v>
@@ -1701,13 +1701,13 @@
         <v>45809</v>
       </c>
       <c r="B73" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C73" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D73" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E73">
         <v>16812346</v>
@@ -1718,13 +1718,13 @@
         <v>45809</v>
       </c>
       <c r="B74" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D74" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E74">
         <v>7430</v>
@@ -1735,13 +1735,13 @@
         <v>45809</v>
       </c>
       <c r="B75" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D75" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E75">
         <v>30389</v>
@@ -1752,13 +1752,13 @@
         <v>45809</v>
       </c>
       <c r="B76" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C76" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D76" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E76">
         <v>6925044</v>
@@ -1769,13 +1769,13 @@
         <v>45809</v>
       </c>
       <c r="B77" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C77" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D77" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E77">
         <v>177118</v>
@@ -1786,13 +1786,13 @@
         <v>45809</v>
       </c>
       <c r="B78" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C78" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D78" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E78">
         <v>535901</v>
@@ -1803,13 +1803,13 @@
         <v>45809</v>
       </c>
       <c r="B79" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D79" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E79">
         <v>369596</v>
@@ -1820,13 +1820,13 @@
         <v>45809</v>
       </c>
       <c r="B80" t="s">
+        <v>13</v>
+      </c>
+      <c r="C80" t="s">
         <v>14</v>
       </c>
-      <c r="C80" t="s">
-        <v>15</v>
-      </c>
       <c r="D80" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E80">
         <v>424562</v>
@@ -1837,13 +1837,13 @@
         <v>45809</v>
       </c>
       <c r="B81" t="s">
+        <v>13</v>
+      </c>
+      <c r="C81" t="s">
         <v>14</v>
       </c>
-      <c r="C81" t="s">
-        <v>15</v>
-      </c>
       <c r="D81" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E81">
         <v>1289856</v>
@@ -1854,13 +1854,13 @@
         <v>45809</v>
       </c>
       <c r="B82" t="s">
+        <v>13</v>
+      </c>
+      <c r="C82" t="s">
         <v>14</v>
       </c>
-      <c r="C82" t="s">
-        <v>15</v>
-      </c>
       <c r="D82" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E82">
         <v>2819216</v>
@@ -1871,13 +1871,13 @@
         <v>45809</v>
       </c>
       <c r="B83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C83" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D83" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E83">
         <v>492854</v>
@@ -1888,13 +1888,13 @@
         <v>45809</v>
       </c>
       <c r="B84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C84" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D84" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E84">
         <v>842965</v>
@@ -1905,13 +1905,13 @@
         <v>45809</v>
       </c>
       <c r="B85" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C85" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D85" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E85">
         <v>13029618</v>
@@ -1922,13 +1922,13 @@
         <v>45839</v>
       </c>
       <c r="B86" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" t="s">
         <v>5</v>
       </c>
-      <c r="C86" t="s">
-        <v>6</v>
-      </c>
       <c r="D86" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E86">
         <v>583256</v>
@@ -1939,13 +1939,13 @@
         <v>45839</v>
       </c>
       <c r="B87" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" t="s">
         <v>5</v>
       </c>
-      <c r="C87" t="s">
-        <v>6</v>
-      </c>
       <c r="D87" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E87">
         <v>978535</v>
@@ -1956,13 +1956,13 @@
         <v>45839</v>
       </c>
       <c r="B88" t="s">
+        <v>4</v>
+      </c>
+      <c r="C88" t="s">
         <v>5</v>
       </c>
-      <c r="C88" t="s">
-        <v>6</v>
-      </c>
       <c r="D88" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E88">
         <v>3009366</v>
@@ -1973,13 +1973,13 @@
         <v>45839</v>
       </c>
       <c r="B89" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C89" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D89" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E89">
         <v>1027683</v>
@@ -1990,13 +1990,13 @@
         <v>45839</v>
       </c>
       <c r="B90" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C90" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D90" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E90">
         <v>5104157</v>
@@ -2007,13 +2007,13 @@
         <v>45839</v>
       </c>
       <c r="B91" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C91" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D91" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E91">
         <v>12733084</v>
@@ -2024,13 +2024,13 @@
         <v>45839</v>
       </c>
       <c r="B92" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C92" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D92" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E92">
         <v>928144</v>
@@ -2041,13 +2041,13 @@
         <v>45839</v>
       </c>
       <c r="B93" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C93" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D93" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E93">
         <v>3071240</v>
@@ -2058,13 +2058,13 @@
         <v>45839</v>
       </c>
       <c r="B94" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C94" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D94" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E94">
         <v>16704551</v>
@@ -2075,13 +2075,13 @@
         <v>45839</v>
       </c>
       <c r="B95" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C95" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D95" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E95">
         <v>7534</v>
@@ -2092,13 +2092,13 @@
         <v>45839</v>
       </c>
       <c r="B96" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C96" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D96" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E96">
         <v>33640</v>
@@ -2109,13 +2109,13 @@
         <v>45839</v>
       </c>
       <c r="B97" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C97" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D97" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E97">
         <v>6801221</v>
@@ -2126,13 +2126,13 @@
         <v>45839</v>
       </c>
       <c r="B98" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C98" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D98" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E98">
         <v>174980</v>
@@ -2143,13 +2143,13 @@
         <v>45839</v>
       </c>
       <c r="B99" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C99" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D99" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E99">
         <v>529902</v>
@@ -2160,13 +2160,13 @@
         <v>45839</v>
       </c>
       <c r="B100" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C100" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D100" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E100">
         <v>376015</v>
@@ -2177,13 +2177,13 @@
         <v>45839</v>
       </c>
       <c r="B101" t="s">
+        <v>13</v>
+      </c>
+      <c r="C101" t="s">
         <v>14</v>
       </c>
-      <c r="C101" t="s">
-        <v>15</v>
-      </c>
       <c r="D101" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E101">
         <v>424033</v>
@@ -2194,13 +2194,13 @@
         <v>45839</v>
       </c>
       <c r="B102" t="s">
+        <v>13</v>
+      </c>
+      <c r="C102" t="s">
         <v>14</v>
       </c>
-      <c r="C102" t="s">
-        <v>15</v>
-      </c>
       <c r="D102" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E102">
         <v>1271953</v>
@@ -2211,13 +2211,13 @@
         <v>45839</v>
       </c>
       <c r="B103" t="s">
+        <v>13</v>
+      </c>
+      <c r="C103" t="s">
         <v>14</v>
       </c>
-      <c r="C103" t="s">
-        <v>15</v>
-      </c>
       <c r="D103" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E103">
         <v>2767046</v>
@@ -2228,13 +2228,13 @@
         <v>45839</v>
       </c>
       <c r="B104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C104" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D104" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E104">
         <v>494871</v>
@@ -2245,13 +2245,13 @@
         <v>45839</v>
       </c>
       <c r="B105" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C105" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D105" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E105">
         <v>848378</v>
@@ -2262,13 +2262,13 @@
         <v>45839</v>
       </c>
       <c r="B106" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C106" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D106" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E106">
         <v>13905102</v>
@@ -2279,13 +2279,13 @@
         <v>45870</v>
       </c>
       <c r="B107" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107" t="s">
         <v>5</v>
       </c>
-      <c r="C107" t="s">
-        <v>6</v>
-      </c>
       <c r="D107" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E107">
         <v>576113</v>
@@ -2296,13 +2296,13 @@
         <v>45870</v>
       </c>
       <c r="B108" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108" t="s">
         <v>5</v>
       </c>
-      <c r="C108" t="s">
-        <v>6</v>
-      </c>
       <c r="D108" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E108">
         <v>968490</v>
@@ -2313,13 +2313,13 @@
         <v>45870</v>
       </c>
       <c r="B109" t="s">
+        <v>4</v>
+      </c>
+      <c r="C109" t="s">
         <v>5</v>
       </c>
-      <c r="C109" t="s">
-        <v>6</v>
-      </c>
       <c r="D109" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E109">
         <v>3007934</v>
@@ -2330,13 +2330,13 @@
         <v>45870</v>
       </c>
       <c r="B110" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C110" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D110" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E110">
         <v>1054746</v>
@@ -2347,13 +2347,13 @@
         <v>45870</v>
       </c>
       <c r="B111" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C111" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D111" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E111">
         <v>4865521</v>
@@ -2364,13 +2364,13 @@
         <v>45870</v>
       </c>
       <c r="B112" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C112" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D112" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E112">
         <v>12932384</v>
@@ -2381,13 +2381,13 @@
         <v>45870</v>
       </c>
       <c r="B113" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C113" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D113" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E113">
         <v>904119</v>
@@ -2398,13 +2398,13 @@
         <v>45870</v>
       </c>
       <c r="B114" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C114" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D114" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E114">
         <v>3349681</v>
@@ -2415,13 +2415,13 @@
         <v>45870</v>
       </c>
       <c r="B115" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C115" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D115" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E115">
         <v>16782365</v>
@@ -2432,13 +2432,13 @@
         <v>45870</v>
       </c>
       <c r="B116" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C116" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D116" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E116">
         <v>7347</v>
@@ -2449,13 +2449,13 @@
         <v>45870</v>
       </c>
       <c r="B117" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C117" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D117" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E117">
         <v>0</v>
@@ -2466,13 +2466,13 @@
         <v>45870</v>
       </c>
       <c r="B118" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C118" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D118" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E118">
         <v>7003306</v>
@@ -2483,13 +2483,13 @@
         <v>45870</v>
       </c>
       <c r="B119" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C119" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D119" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E119">
         <v>178582</v>
@@ -2500,13 +2500,13 @@
         <v>45870</v>
       </c>
       <c r="B120" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C120" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D120" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E120">
         <v>540261</v>
@@ -2517,13 +2517,13 @@
         <v>45870</v>
       </c>
       <c r="B121" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C121" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D121" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E121">
         <v>365085</v>
@@ -2534,13 +2534,13 @@
         <v>45870</v>
       </c>
       <c r="B122" t="s">
+        <v>13</v>
+      </c>
+      <c r="C122" t="s">
         <v>14</v>
       </c>
-      <c r="C122" t="s">
-        <v>15</v>
-      </c>
       <c r="D122" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E122">
         <v>426339</v>
@@ -2551,13 +2551,13 @@
         <v>45870</v>
       </c>
       <c r="B123" t="s">
+        <v>13</v>
+      </c>
+      <c r="C123" t="s">
         <v>14</v>
       </c>
-      <c r="C123" t="s">
-        <v>15</v>
-      </c>
       <c r="D123" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E123">
         <v>1300319</v>
@@ -2568,13 +2568,13 @@
         <v>45870</v>
       </c>
       <c r="B124" t="s">
+        <v>13</v>
+      </c>
+      <c r="C124" t="s">
         <v>14</v>
       </c>
-      <c r="C124" t="s">
-        <v>15</v>
-      </c>
       <c r="D124" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E124">
         <v>2868038</v>
@@ -2585,13 +2585,13 @@
         <v>45870</v>
       </c>
       <c r="B125" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C125" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D125" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E125">
         <v>464818</v>
@@ -2602,13 +2602,13 @@
         <v>45870</v>
       </c>
       <c r="B126" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C126" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D126" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E126">
         <v>785881</v>
@@ -2619,13 +2619,13 @@
         <v>45870</v>
       </c>
       <c r="B127" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C127" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D127" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E127">
         <v>13296517</v>
@@ -2636,13 +2636,13 @@
         <v>45901</v>
       </c>
       <c r="B128" t="s">
+        <v>4</v>
+      </c>
+      <c r="C128" t="s">
         <v>5</v>
       </c>
-      <c r="C128" t="s">
-        <v>6</v>
-      </c>
       <c r="D128" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E128">
         <v>595296</v>
@@ -2653,13 +2653,13 @@
         <v>45901</v>
       </c>
       <c r="B129" t="s">
+        <v>4</v>
+      </c>
+      <c r="C129" t="s">
         <v>5</v>
       </c>
-      <c r="C129" t="s">
-        <v>6</v>
-      </c>
       <c r="D129" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E129">
         <v>951527</v>
@@ -2670,13 +2670,13 @@
         <v>45901</v>
       </c>
       <c r="B130" t="s">
+        <v>4</v>
+      </c>
+      <c r="C130" t="s">
         <v>5</v>
       </c>
-      <c r="C130" t="s">
-        <v>6</v>
-      </c>
       <c r="D130" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E130">
         <v>3005914</v>
@@ -2687,13 +2687,13 @@
         <v>45901</v>
       </c>
       <c r="B131" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C131" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D131" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E131">
         <v>1055685</v>
@@ -2704,13 +2704,13 @@
         <v>45901</v>
       </c>
       <c r="B132" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C132" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D132" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E132">
         <v>4768701</v>
@@ -2721,13 +2721,13 @@
         <v>45901</v>
       </c>
       <c r="B133" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C133" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D133" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E133">
         <v>13057256</v>
@@ -2738,13 +2738,13 @@
         <v>45901</v>
       </c>
       <c r="B134" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C134" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D134" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E134">
         <v>938615</v>
@@ -2755,13 +2755,13 @@
         <v>45901</v>
       </c>
       <c r="B135" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C135" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D135" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E135">
         <v>3329054</v>
@@ -2772,13 +2772,13 @@
         <v>45901</v>
       </c>
       <c r="B136" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C136" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D136" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E136">
         <v>16920687</v>
@@ -2789,13 +2789,13 @@
         <v>45901</v>
       </c>
       <c r="B137" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C137" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D137" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E137">
         <v>7317</v>
@@ -2806,13 +2806,13 @@
         <v>45901</v>
       </c>
       <c r="B138" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C138" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D138" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E138">
         <v>0</v>
@@ -2823,13 +2823,13 @@
         <v>45901</v>
       </c>
       <c r="B139" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C139" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D139" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E139">
         <v>7071965</v>
@@ -2840,13 +2840,13 @@
         <v>45901</v>
       </c>
       <c r="B140" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C140" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D140" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E140">
         <v>177088</v>
@@ -2857,13 +2857,13 @@
         <v>45901</v>
       </c>
       <c r="B141" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C141" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D141" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E141">
         <v>542123</v>
@@ -2874,13 +2874,13 @@
         <v>45901</v>
       </c>
       <c r="B142" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C142" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D142" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E142">
         <v>360997</v>
@@ -2891,13 +2891,13 @@
         <v>45901</v>
       </c>
       <c r="B143" t="s">
+        <v>13</v>
+      </c>
+      <c r="C143" t="s">
         <v>14</v>
       </c>
-      <c r="C143" t="s">
-        <v>15</v>
-      </c>
       <c r="D143" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E143">
         <v>419220</v>
@@ -2908,13 +2908,13 @@
         <v>45901</v>
       </c>
       <c r="B144" t="s">
+        <v>13</v>
+      </c>
+      <c r="C144" t="s">
         <v>14</v>
       </c>
-      <c r="C144" t="s">
-        <v>15</v>
-      </c>
       <c r="D144" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E144">
         <v>1306051</v>
@@ -2925,13 +2925,13 @@
         <v>45901</v>
       </c>
       <c r="B145" t="s">
+        <v>13</v>
+      </c>
+      <c r="C145" t="s">
         <v>14</v>
       </c>
-      <c r="C145" t="s">
-        <v>15</v>
-      </c>
       <c r="D145" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E145">
         <v>2872213</v>
@@ -2942,13 +2942,13 @@
         <v>45901</v>
       </c>
       <c r="B146" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C146" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D146" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E146">
         <v>468903</v>
@@ -2959,13 +2959,13 @@
         <v>45901</v>
       </c>
       <c r="B147" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C147" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D147" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E147">
         <v>791441</v>
@@ -2976,13 +2976,13 @@
         <v>45901</v>
       </c>
       <c r="B148" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C148" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D148" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E148">
         <v>13519895</v>
@@ -2993,13 +2993,13 @@
         <v>45931</v>
       </c>
       <c r="B149" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C149" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D149" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E149">
         <v>1073720</v>
@@ -3010,13 +3010,13 @@
         <v>45931</v>
       </c>
       <c r="B150" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C150" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D150" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E150">
         <v>4649138</v>
@@ -3027,13 +3027,13 @@
         <v>45931</v>
       </c>
       <c r="B151" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C151" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D151" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E151">
         <v>13114187</v>
@@ -3044,13 +3044,13 @@
         <v>45931</v>
       </c>
       <c r="B152" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C152" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D152" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E152">
         <v>1073720</v>
@@ -3061,13 +3061,13 @@
         <v>45931</v>
       </c>
       <c r="B153" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C153" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D153" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E153">
         <v>4649138</v>
@@ -3078,13 +3078,13 @@
         <v>45931</v>
       </c>
       <c r="B154" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C154" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D154" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E154">
         <v>13114187</v>
@@ -3095,13 +3095,13 @@
         <v>45931</v>
       </c>
       <c r="B155" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C155" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D155" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E155">
         <v>958866</v>
@@ -3112,13 +3112,13 @@
         <v>45931</v>
       </c>
       <c r="B156" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C156" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D156" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E156">
         <v>3160567</v>
@@ -3129,13 +3129,13 @@
         <v>45931</v>
       </c>
       <c r="B157" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C157" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D157" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E157">
         <v>17136713</v>
@@ -3146,13 +3146,13 @@
         <v>45931</v>
       </c>
       <c r="B158" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C158" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D158" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E158">
         <v>7285</v>
@@ -3163,13 +3163,13 @@
         <v>45931</v>
       </c>
       <c r="B159" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C159" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D159" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E159">
         <v>0</v>
@@ -3180,13 +3180,13 @@
         <v>45931</v>
       </c>
       <c r="B160" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C160" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D160" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E160">
         <v>7118868</v>
@@ -3197,13 +3197,13 @@
         <v>45931</v>
       </c>
       <c r="B161" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C161" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D161" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E161">
         <v>177817</v>
@@ -3214,13 +3214,13 @@
         <v>45931</v>
       </c>
       <c r="B162" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C162" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D162" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E162">
         <v>543934</v>
@@ -3231,13 +3231,13 @@
         <v>45931</v>
       </c>
       <c r="B163" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C163" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D163" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E163">
         <v>358616</v>
@@ -3248,13 +3248,13 @@
         <v>45931</v>
       </c>
       <c r="B164" t="s">
+        <v>13</v>
+      </c>
+      <c r="C164" t="s">
         <v>14</v>
       </c>
-      <c r="C164" t="s">
-        <v>15</v>
-      </c>
       <c r="D164" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E164">
         <v>420631</v>
@@ -3265,13 +3265,13 @@
         <v>45931</v>
       </c>
       <c r="B165" t="s">
+        <v>13</v>
+      </c>
+      <c r="C165" t="s">
         <v>14</v>
       </c>
-      <c r="C165" t="s">
-        <v>15</v>
-      </c>
       <c r="D165" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E165">
         <v>1312257</v>
@@ -3282,13 +3282,13 @@
         <v>45931</v>
       </c>
       <c r="B166" t="s">
+        <v>13</v>
+      </c>
+      <c r="C166" t="s">
         <v>14</v>
       </c>
-      <c r="C166" t="s">
-        <v>15</v>
-      </c>
       <c r="D166" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E166">
         <v>2903178</v>
@@ -3299,13 +3299,13 @@
         <v>45931</v>
       </c>
       <c r="B167" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C167" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D167" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E167">
         <v>478799</v>
@@ -3316,13 +3316,13 @@
         <v>45931</v>
       </c>
       <c r="B168" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C168" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D168" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E168">
         <v>880424</v>
@@ -3333,13 +3333,13 @@
         <v>45931</v>
       </c>
       <c r="B169" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C169" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D169" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E169">
         <v>13511787</v>
@@ -3350,13 +3350,13 @@
         <v>45962</v>
       </c>
       <c r="B170" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C170" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D170" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E170">
         <v>1075803</v>
@@ -3367,13 +3367,13 @@
         <v>45962</v>
       </c>
       <c r="B171" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C171" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D171" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E171">
         <v>4737327</v>
@@ -3384,13 +3384,13 @@
         <v>45962</v>
       </c>
       <c r="B172" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C172" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D172" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E172">
         <v>12984482</v>
@@ -3401,13 +3401,13 @@
         <v>45962</v>
       </c>
       <c r="B173" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C173" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D173" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E173">
         <v>1075803</v>
@@ -3418,13 +3418,13 @@
         <v>45962</v>
       </c>
       <c r="B174" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C174" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D174" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E174">
         <v>4737327</v>
@@ -3435,13 +3435,13 @@
         <v>45962</v>
       </c>
       <c r="B175" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C175" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D175" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E175">
         <v>12984482</v>
@@ -3452,13 +3452,13 @@
         <v>45962</v>
       </c>
       <c r="B176" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C176" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D176" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E176">
         <v>920861</v>
@@ -3469,13 +3469,13 @@
         <v>45962</v>
       </c>
       <c r="B177" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C177" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D177" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E177">
         <v>3192609</v>
@@ -3486,13 +3486,13 @@
         <v>45962</v>
       </c>
       <c r="B178" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C178" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D178" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E178">
         <v>17205622</v>
@@ -3503,13 +3503,13 @@
         <v>45962</v>
       </c>
       <c r="B179" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C179" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D179" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E179">
         <v>7250</v>
@@ -3520,13 +3520,13 @@
         <v>45962</v>
       </c>
       <c r="B180" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C180" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D180" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E180">
         <v>0</v>
@@ -3537,13 +3537,13 @@
         <v>45962</v>
       </c>
       <c r="B181" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C181" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D181" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E181">
         <v>7217711</v>
@@ -3554,13 +3554,13 @@
         <v>45962</v>
       </c>
       <c r="B182" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C182" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D182" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E182">
         <v>178567</v>
@@ -3571,13 +3571,13 @@
         <v>45962</v>
       </c>
       <c r="B183" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C183" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D183" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E183">
         <v>544870</v>
@@ -3588,13 +3588,13 @@
         <v>45962</v>
       </c>
       <c r="B184" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C184" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D184" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E184">
         <v>357695</v>
@@ -3605,13 +3605,13 @@
         <v>45962</v>
       </c>
       <c r="B185" t="s">
+        <v>13</v>
+      </c>
+      <c r="C185" t="s">
         <v>14</v>
       </c>
-      <c r="C185" t="s">
-        <v>15</v>
-      </c>
       <c r="D185" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E185">
         <v>420199</v>
@@ -3622,13 +3622,13 @@
         <v>45962</v>
       </c>
       <c r="B186" t="s">
+        <v>13</v>
+      </c>
+      <c r="C186" t="s">
         <v>14</v>
       </c>
-      <c r="C186" t="s">
-        <v>15</v>
-      </c>
       <c r="D186" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E186">
         <v>1318401</v>
@@ -3639,13 +3639,13 @@
         <v>45962</v>
       </c>
       <c r="B187" t="s">
+        <v>13</v>
+      </c>
+      <c r="C187" t="s">
         <v>14</v>
       </c>
-      <c r="C187" t="s">
-        <v>15</v>
-      </c>
       <c r="D187" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E187">
         <v>2922882</v>
@@ -3656,13 +3656,13 @@
         <v>45962</v>
       </c>
       <c r="B188" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C188" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D188" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E188">
         <v>459333</v>
@@ -3673,13 +3673,13 @@
         <v>45962</v>
       </c>
       <c r="B189" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C189" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D189" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E189">
         <v>902091</v>
@@ -3690,13 +3690,13 @@
         <v>45962</v>
       </c>
       <c r="B190" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C190" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D190" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E190">
         <v>13616834</v>
@@ -3707,13 +3707,13 @@
         <v>45992</v>
       </c>
       <c r="B191" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C191" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D191" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E191">
         <v>1072126</v>
@@ -3724,13 +3724,13 @@
         <v>45992</v>
       </c>
       <c r="B192" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C192" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D192" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E192">
         <v>4824509</v>
@@ -3741,13 +3741,13 @@
         <v>45992</v>
       </c>
       <c r="B193" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C193" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D193" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E193">
         <v>12846831</v>
@@ -3758,13 +3758,13 @@
         <v>45992</v>
       </c>
       <c r="B194" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C194" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D194" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E194">
         <v>1072126</v>
@@ -3775,13 +3775,13 @@
         <v>45992</v>
       </c>
       <c r="B195" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C195" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D195" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E195">
         <v>4824509</v>
@@ -3792,13 +3792,13 @@
         <v>45992</v>
       </c>
       <c r="B196" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C196" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D196" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E196">
         <v>12846831</v>
@@ -3809,13 +3809,13 @@
         <v>45992</v>
       </c>
       <c r="B197" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C197" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D197" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E197">
         <v>917515</v>
@@ -3826,13 +3826,13 @@
         <v>45992</v>
       </c>
       <c r="B198" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C198" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D198" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E198">
         <v>3224180</v>
@@ -3843,13 +3843,13 @@
         <v>45992</v>
       </c>
       <c r="B199" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C199" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D199" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E199">
         <v>17212550</v>
@@ -3860,13 +3860,13 @@
         <v>45992</v>
       </c>
       <c r="B200" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C200" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D200" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E200">
         <v>7233</v>
@@ -3877,13 +3877,13 @@
         <v>45992</v>
       </c>
       <c r="B201" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C201" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D201" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E201">
         <v>0</v>
@@ -3894,13 +3894,13 @@
         <v>45992</v>
       </c>
       <c r="B202" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C202" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D202" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E202">
         <v>7286283</v>
@@ -3911,13 +3911,13 @@
         <v>45992</v>
       </c>
       <c r="B203" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C203" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D203" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E203">
         <v>190682</v>
@@ -3928,13 +3928,13 @@
         <v>45992</v>
       </c>
       <c r="B204" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C204" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D204" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E204">
         <v>545038</v>
@@ -3945,13 +3945,13 @@
         <v>45992</v>
       </c>
       <c r="B205" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C205" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D205" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E205">
         <v>355670</v>
@@ -3962,13 +3962,13 @@
         <v>45992</v>
       </c>
       <c r="B206" t="s">
+        <v>13</v>
+      </c>
+      <c r="C206" t="s">
         <v>14</v>
       </c>
-      <c r="C206" t="s">
-        <v>15</v>
-      </c>
       <c r="D206" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E206">
         <v>420224</v>
@@ -3979,13 +3979,13 @@
         <v>45992</v>
       </c>
       <c r="B207" t="s">
+        <v>13</v>
+      </c>
+      <c r="C207" t="s">
         <v>14</v>
       </c>
-      <c r="C207" t="s">
-        <v>15</v>
-      </c>
       <c r="D207" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E207">
         <v>1321173</v>
@@ -3996,13 +3996,13 @@
         <v>45992</v>
       </c>
       <c r="B208" t="s">
+        <v>13</v>
+      </c>
+      <c r="C208" t="s">
         <v>14</v>
       </c>
-      <c r="C208" t="s">
-        <v>15</v>
-      </c>
       <c r="D208" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E208">
         <v>2932710</v>
@@ -4013,13 +4013,13 @@
         <v>45992</v>
       </c>
       <c r="B209" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C209" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D209" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E209">
         <v>459389</v>
@@ -4030,13 +4030,13 @@
         <v>45992</v>
       </c>
       <c r="B210" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C210" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D210" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E210">
         <v>918195</v>
@@ -4047,13 +4047,13 @@
         <v>45992</v>
       </c>
       <c r="B211" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C211" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D211" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E211">
         <v>13602756</v>
@@ -4064,13 +4064,13 @@
         <v>46023</v>
       </c>
       <c r="B212" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C212" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D212" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E212">
         <v>1068145</v>
@@ -4081,13 +4081,13 @@
         <v>46023</v>
       </c>
       <c r="B213" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C213" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D213" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E213">
         <v>4712374</v>
@@ -4098,13 +4098,13 @@
         <v>46023</v>
       </c>
       <c r="B214" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C214" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D214" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E214">
         <v>12895881</v>
@@ -4115,13 +4115,13 @@
         <v>46023</v>
       </c>
       <c r="B215" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C215" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D215" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E215">
         <v>1068145</v>
@@ -4132,13 +4132,13 @@
         <v>46023</v>
       </c>
       <c r="B216" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C216" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D216" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E216">
         <v>4712374</v>
@@ -4149,13 +4149,13 @@
         <v>46023</v>
       </c>
       <c r="B217" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C217" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D217" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E217">
         <v>12895881</v>
@@ -4166,13 +4166,13 @@
         <v>46023</v>
       </c>
       <c r="B218" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C218" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D218" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E218">
         <v>911238</v>
@@ -4183,13 +4183,13 @@
         <v>46023</v>
       </c>
       <c r="B219" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C219" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D219" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E219">
         <v>3214799</v>
@@ -4200,13 +4200,13 @@
         <v>46023</v>
       </c>
       <c r="B220" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C220" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D220" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E220">
         <v>17183162</v>
@@ -4217,13 +4217,13 @@
         <v>46023</v>
       </c>
       <c r="B221" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C221" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D221" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E221">
         <v>7183</v>
@@ -4234,13 +4234,13 @@
         <v>46023</v>
       </c>
       <c r="B222" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C222" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D222" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E222">
         <v>0</v>
@@ -4251,13 +4251,13 @@
         <v>46023</v>
       </c>
       <c r="B223" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C223" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D223" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E223">
         <v>7294697</v>
@@ -4268,13 +4268,13 @@
         <v>46023</v>
       </c>
       <c r="B224" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C224" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D224" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E224">
         <v>190352</v>
@@ -4285,13 +4285,13 @@
         <v>46023</v>
       </c>
       <c r="B225" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C225" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D225" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E225">
         <v>544333</v>
@@ -4302,13 +4302,13 @@
         <v>46023</v>
       </c>
       <c r="B226" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C226" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D226" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E226">
         <v>353707</v>
@@ -4319,13 +4319,13 @@
         <v>46023</v>
       </c>
       <c r="B227" t="s">
+        <v>13</v>
+      </c>
+      <c r="C227" t="s">
         <v>14</v>
       </c>
-      <c r="C227" t="s">
-        <v>15</v>
-      </c>
       <c r="D227" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E227">
         <v>419159</v>
@@ -4336,13 +4336,13 @@
         <v>46023</v>
       </c>
       <c r="B228" t="s">
+        <v>13</v>
+      </c>
+      <c r="C228" t="s">
         <v>14</v>
       </c>
-      <c r="C228" t="s">
-        <v>15</v>
-      </c>
       <c r="D228" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E228">
         <v>1314627</v>
@@ -4353,13 +4353,13 @@
         <v>46023</v>
       </c>
       <c r="B229" t="s">
+        <v>13</v>
+      </c>
+      <c r="C229" t="s">
         <v>14</v>
       </c>
-      <c r="C229" t="s">
-        <v>15</v>
-      </c>
       <c r="D229" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E229">
         <v>2939095</v>
@@ -4370,13 +4370,13 @@
         <v>46023</v>
       </c>
       <c r="B230" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C230" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D230" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E230">
         <v>460025</v>
@@ -4387,13 +4387,13 @@
         <v>46023</v>
       </c>
       <c r="B231" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C231" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D231" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E231">
         <v>912034</v>
@@ -4404,13 +4404,13 @@
         <v>46023</v>
       </c>
       <c r="B232" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C232" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D232" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E232">
         <v>13443890</v>
@@ -4421,13 +4421,13 @@
         <v>46054</v>
       </c>
       <c r="B233" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C233" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D233" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E233">
         <v>1065291</v>
@@ -4438,13 +4438,13 @@
         <v>46054</v>
       </c>
       <c r="B234" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C234" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D234" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E234">
         <v>4706667</v>
@@ -4455,13 +4455,13 @@
         <v>46054</v>
       </c>
       <c r="B235" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C235" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D235" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E235">
         <v>12848693</v>
@@ -4472,13 +4472,13 @@
         <v>46054</v>
       </c>
       <c r="B236" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C236" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D236" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E236">
         <v>1065291</v>
@@ -4489,13 +4489,13 @@
         <v>46054</v>
       </c>
       <c r="B237" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C237" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D237" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E237">
         <v>4706667</v>
@@ -4506,13 +4506,13 @@
         <v>46054</v>
       </c>
       <c r="B238" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C238" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D238" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E238">
         <v>12848693</v>
@@ -4523,13 +4523,13 @@
         <v>46054</v>
       </c>
       <c r="B239" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C239" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D239" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E239">
         <v>905208</v>
@@ -4540,13 +4540,13 @@
         <v>46054</v>
       </c>
       <c r="B240" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C240" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D240" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E240">
         <v>3118487</v>
@@ -4557,13 +4557,13 @@
         <v>46054</v>
       </c>
       <c r="B241" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C241" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D241" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E241">
         <v>17299267</v>
@@ -4574,13 +4574,13 @@
         <v>46054</v>
       </c>
       <c r="B242" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C242" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D242" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E242">
         <v>7169</v>
@@ -4591,13 +4591,13 @@
         <v>46054</v>
       </c>
       <c r="B243" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C243" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D243" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E243">
         <v>0</v>
@@ -4608,13 +4608,13 @@
         <v>46054</v>
       </c>
       <c r="B244" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C244" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D244" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E244">
         <v>7358463</v>
@@ -4625,13 +4625,13 @@
         <v>46054</v>
       </c>
       <c r="B245" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C245" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D245" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E245">
         <v>190391</v>
@@ -4642,13 +4642,13 @@
         <v>46054</v>
       </c>
       <c r="B246" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C246" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D246" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E246">
         <v>545203</v>
@@ -4659,13 +4659,13 @@
         <v>46054</v>
       </c>
       <c r="B247" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C247" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D247" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E247">
         <v>345658</v>
@@ -4676,13 +4676,13 @@
         <v>46054</v>
       </c>
       <c r="B248" t="s">
+        <v>13</v>
+      </c>
+      <c r="C248" t="s">
         <v>14</v>
       </c>
-      <c r="C248" t="s">
-        <v>15</v>
-      </c>
       <c r="D248" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E248">
         <v>416511</v>
@@ -4693,13 +4693,13 @@
         <v>46054</v>
       </c>
       <c r="B249" t="s">
+        <v>13</v>
+      </c>
+      <c r="C249" t="s">
         <v>14</v>
       </c>
-      <c r="C249" t="s">
-        <v>15</v>
-      </c>
       <c r="D249" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E249">
         <v>1314467</v>
@@ -4710,13 +4710,13 @@
         <v>46054</v>
       </c>
       <c r="B250" t="s">
+        <v>13</v>
+      </c>
+      <c r="C250" t="s">
         <v>14</v>
       </c>
-      <c r="C250" t="s">
-        <v>15</v>
-      </c>
       <c r="D250" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E250">
         <v>2937383</v>
@@ -4727,13 +4727,13 @@
         <v>46054</v>
       </c>
       <c r="B251" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C251" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D251" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E251">
         <v>461281</v>
@@ -4744,13 +4744,13 @@
         <v>46054</v>
       </c>
       <c r="B252" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C252" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D252" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E252">
         <v>895107</v>
@@ -4761,13 +4761,13 @@
         <v>46054</v>
       </c>
       <c r="B253" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C253" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D253" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E253">
         <v>13598741</v>

</xml_diff>